<commit_message>
Add first Asia model with BAU scenario parameterization
Include the first model for ASIA region with its full parameterization:
- Update configuration files (Config_MOMF_T1_A, Config_country_codes, Config_region_consolidation)
- Update OG_csvs_inputs with Asia region data across all OSeMOSYS parameters
- Add BAU scenario outputs (A1_Outputs, A2_Outputs_Params_otoole/BAU)
- Add completed parameterization files (A-O_*_COMPLETED.xlsx)
- Update A2_Extra_Inputs (Emissions, Storage) and Tech_Country_Matrix
- Remove old NDC/NDC+ELC/NDC_NoRPO scenario outputs and Old_Inputs folder
- Update dvc.lock
</commit_message>
<xml_diff>
--- a/t1_confection/A2_Extra_Inputs/A-Xtra_Emissions.xlsx
+++ b/t1_confection/A2_Extra_Inputs/A-Xtra_Emissions.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E138"/>
+  <dimension ref="A1:E113"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="19.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -486,16 +486,16 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PWRCOAARGXX</t>
+          <t>PWRCCSBGDXX</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CO2ARG</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.2734</v>
+        <v>0.0273</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -509,16 +509,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PWRCOAARGXX</t>
+          <t>PWRCCSBGDXX</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CO2ARG</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.2734</v>
+        <v>0.0273</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -532,16 +532,16 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PWRCOABRAXX</t>
+          <t>PWRCCSINDEA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CO2BRA</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.2752</v>
+        <v>0.0273</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -555,16 +555,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PWRCOABRAXX</t>
+          <t>PWRCCSINDEA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CO2BRA</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.2752</v>
+        <v>0.0273</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -578,16 +578,16 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PWRCOACHLXX</t>
+          <t>PWRCCSINDNE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CO2CHL</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.2743</v>
+        <v>0.0273</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -601,16 +601,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PWRCOACHLXX</t>
+          <t>PWRCCSINDNE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CO2CHL</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.2743</v>
+        <v>0.0273</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -624,16 +624,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PWRCOACOLXX</t>
+          <t>PWRCCSINDNO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CO2COL</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.2734</v>
+        <v>0.0273</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -647,16 +647,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PWRCOACOLXX</t>
+          <t>PWRCCSINDNO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CO2COL</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.2734</v>
+        <v>0.0273</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -670,16 +670,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PWRCOADOMXX</t>
+          <t>PWRCCSINDSO</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CO2DOM</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.2762</v>
+        <v>0.0273</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -693,16 +693,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PWRCOADOMXX</t>
+          <t>PWRCCSINDSO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CO2DOM</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.2762</v>
+        <v>0.0273</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -716,16 +716,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PWRCOAGTMXX</t>
+          <t>PWRCCSINDWE</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CO2GTM</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.278</v>
+        <v>0.0273</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -739,16 +739,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PWRCOAGTMXX</t>
+          <t>PWRCCSINDWE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CO2GTM</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.278</v>
+        <v>0.0273</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -762,16 +762,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PWRCOAMEXXX</t>
+          <t>PWRCOABGDXX</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CO2MEX</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.2706</v>
+        <v>0.2724</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -785,16 +785,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PWRCOAMEXXX</t>
+          <t>PWRCOABGDXX</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CO2MEX</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.2706</v>
+        <v>0.2724</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -808,16 +808,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PWRCOAPANXX</t>
+          <t>PWRCOAINDEA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CO2PAN</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.2771</v>
+        <v>0.2715</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -831,16 +831,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PWRCOAPANXX</t>
+          <t>PWRCOAINDEA</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CO2PAN</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.2771</v>
+        <v>0.2715</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -854,16 +854,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PWRCOAPERXX</t>
+          <t>PWRCOAINDNE</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CO2PER</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.278</v>
+        <v>0.2724</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -877,16 +877,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PWRCOAPERXX</t>
+          <t>PWRCOAINDNE</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CO2PER</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.278</v>
+        <v>0.2724</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -900,16 +900,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PWRNGSARGXX</t>
+          <t>PWRCOAINDNO</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CO2ARG</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.12215</v>
+        <v>0.2743</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -923,16 +923,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PWRNGSARGXX</t>
+          <t>PWRCOAINDNO</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CO2ARG</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.12215</v>
+        <v>0.2743</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -946,16 +946,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PWRNGSBOLXX</t>
+          <t>PWRCOAINDSO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CO2BOL</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.12215</v>
+        <v>0.2734</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -969,16 +969,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PWRNGSBOLXX</t>
+          <t>PWRCOAINDSO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CO2BOL</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.12215</v>
+        <v>0.2734</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -992,16 +992,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PWRNGSBRAXX</t>
+          <t>PWRCOAINDWE</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CO2BRA</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.12215</v>
+        <v>0.2743</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1015,16 +1015,16 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PWRNGSBRAXX</t>
+          <t>PWRCOAINDWE</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>CO2BRA</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.12215</v>
+        <v>0.2743</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1038,16 +1038,16 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PWRNGSCHLXX</t>
+          <t>PWRCOALKAXX</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>CO2CHL</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.12215</v>
+        <v>0.2743</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1061,16 +1061,16 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PWRNGSCHLXX</t>
+          <t>PWRCOALKAXX</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CO2CHL</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.12215</v>
+        <v>0.2743</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1084,16 +1084,16 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PWRNGSCOLXX</t>
+          <t>PWRCOGBGDXX</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>CO2COL</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.12215</v>
+        <v>0.2724</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1107,16 +1107,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PWRNGSCOLXX</t>
+          <t>PWRCOGBGDXX</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>CO2COL</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.12215</v>
+        <v>0.2724</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1130,16 +1130,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PWRNGSDOMXX</t>
+          <t>PWRCOGINDEA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>CO2DOM</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.12215</v>
+        <v>0.2724</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1153,16 +1153,16 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PWRNGSDOMXX</t>
+          <t>PWRCOGINDEA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CO2DOM</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.12215</v>
+        <v>0.2724</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1176,16 +1176,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PWRNGSECUXX</t>
+          <t>PWRCOGINDNE</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>CO2ECU</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.12215</v>
+        <v>0.2724</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1199,16 +1199,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PWRNGSECUXX</t>
+          <t>PWRCOGINDNE</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>CO2ECU</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.12215</v>
+        <v>0.2724</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1222,16 +1222,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PWRNGSGTMXX</t>
+          <t>PWRCOGINDNO</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CO2GTM</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.12215</v>
+        <v>0.2724</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1245,16 +1245,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PWRNGSGTMXX</t>
+          <t>PWRCOGINDNO</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>CO2GTM</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.12215</v>
+        <v>0.2724</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1268,16 +1268,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PWRNGSMEXXX</t>
+          <t>PWRCOGINDSO</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CO2MEX</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.12215</v>
+        <v>0.2724</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1291,16 +1291,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PWRNGSMEXXX</t>
+          <t>PWRCOGINDSO</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>CO2MEX</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.12215</v>
+        <v>0.2724</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1314,16 +1314,16 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PWRNGSPANXX</t>
+          <t>PWRCOGINDWE</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CO2PAN</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.12215</v>
+        <v>0.2724</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1337,16 +1337,16 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PWRNGSPANXX</t>
+          <t>PWRCOGINDWE</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CO2PAN</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.12215</v>
+        <v>0.2724</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1360,16 +1360,16 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PWRNGSPERXX</t>
+          <t>PWRCOGLKAXX</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CO2PER</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.12215</v>
+        <v>0.2724</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1383,16 +1383,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PWRNGSPERXX</t>
+          <t>PWRCOGLKAXX</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CO2PER</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.12215</v>
+        <v>0.2724</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1406,12 +1406,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PWRNGSSLVXX</t>
+          <t>PWRNGSBGDXX</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CO2SLV</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1429,12 +1429,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PWRNGSSLVXX</t>
+          <t>PWRNGSBGDXX</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>CO2SLV</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1452,16 +1452,16 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PWROILARGXX</t>
+          <t>PWRNGSINDEA</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CO2ARG</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.2212</v>
+        <v>0.12215</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1475,16 +1475,16 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PWROILARGXX</t>
+          <t>PWRNGSINDEA</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>CO2ARG</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.2212</v>
+        <v>0.12215</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1498,16 +1498,16 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PWROILBOLXX</t>
+          <t>PWRNGSINDNE</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>CO2BOL</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.2177</v>
+        <v>0.12215</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1521,16 +1521,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PWROILBOLXX</t>
+          <t>PWRNGSINDNE</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CO2BOL</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.2177</v>
+        <v>0.12215</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1544,16 +1544,16 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PWROILBRAXX</t>
+          <t>PWRNGSINDNO</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>CO2BRA</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.2223285714285714</v>
+        <v>0.12215</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1567,16 +1567,16 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PWROILBRAXX</t>
+          <t>PWRNGSINDNO</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>CO2BRA</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.2223285714285714</v>
+        <v>0.12215</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1590,16 +1590,16 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PWROILBRBXX</t>
+          <t>PWRNGSINDSO</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>CO2BRB</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.1971</v>
+        <v>0.12215</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1613,16 +1613,16 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PWROILBRBXX</t>
+          <t>PWRNGSINDSO</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>CO2BRB</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.1971</v>
+        <v>0.12215</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1636,16 +1636,16 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PWROILCHLXX</t>
+          <t>PWRNGSINDWE</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>CO2CHL</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.2155</v>
+        <v>0.12215</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1659,16 +1659,16 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PWROILCHLXX</t>
+          <t>PWRNGSINDWE</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>CO2CHL</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.2155</v>
+        <v>0.12215</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1682,16 +1682,16 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PWROILCOLXX</t>
+          <t>PWRNGSLKAXX</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>CO2COL</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.195</v>
+        <v>0.12215</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1705,16 +1705,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PWROILCOLXX</t>
+          <t>PWRNGSLKAXX</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>CO2COL</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.195</v>
+        <v>0.12215</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1728,16 +1728,16 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PWROILCRIXX</t>
+          <t>PWROILBGDXX</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>CO2CRI</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.2021</v>
+        <v>0.2042</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1751,16 +1751,16 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PWROILCRIXX</t>
+          <t>PWROILBGDXX</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>CO2CRI</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.2021</v>
+        <v>0.2042</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1774,16 +1774,16 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PWROILDOMXX</t>
+          <t>PWROILINDEA</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>CO2DOM</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.2042</v>
+        <v>0.2177</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1797,16 +1797,16 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>PWROILDOMXX</t>
+          <t>PWROILINDEA</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>CO2DOM</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.2042</v>
+        <v>0.2177</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1820,16 +1820,16 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>PWROILECUXX</t>
+          <t>PWROILINDNE</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>CO2ECU</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.2035</v>
+        <v>0.2177</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1843,16 +1843,16 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PWROILECUXX</t>
+          <t>PWROILINDNE</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>CO2ECU</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.2035</v>
+        <v>0.2177</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1866,16 +1866,16 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PWROILGTMXX</t>
+          <t>PWROILINDNO</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>CO2GTM</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.2092</v>
+        <v>0.195</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1889,16 +1889,16 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PWROILGTMXX</t>
+          <t>PWROILINDNO</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>CO2GTM</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.2092</v>
+        <v>0.195</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1912,16 +1912,16 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>PWROILHNDXX</t>
+          <t>PWROILINDSO</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>CO2HND</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.2063</v>
+        <v>0.1999</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1935,16 +1935,16 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PWROILHNDXX</t>
+          <t>PWROILINDSO</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>CO2HND</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.2063</v>
+        <v>0.1999</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1958,16 +1958,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>PWROILHTIXX</t>
+          <t>PWROILINDWE</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>CO2HTI</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.2177</v>
+        <v>0.2077</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1981,16 +1981,16 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>PWROILHTIXX</t>
+          <t>PWROILINDWE</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>CO2HTI</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.2177</v>
+        <v>0.2077</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2004,16 +2004,16 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PWROILMEXXX</t>
+          <t>PWROILLKAXX</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>CO2MEX</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.2042</v>
+        <v>0.2063</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2027,16 +2027,16 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PWROILMEXXX</t>
+          <t>PWROILLKAXX</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>CO2MEX</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0.2042</v>
+        <v>0.2063</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2050,16 +2050,16 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PWROILNICXX</t>
+          <t>PWROTHBGDXX</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>CO2NIC</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.2063</v>
+        <v>0.0503</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2073,16 +2073,16 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PWROILNICXX</t>
+          <t>PWROTHBGDXX</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>CO2NIC</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.2063</v>
+        <v>0.0503</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2096,16 +2096,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PWROILPANXX</t>
+          <t>PWROTHBTNXX</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>CO2PAN</t>
+          <t>CO2BTN</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.2077</v>
+        <v>0.0503</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2119,16 +2119,16 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PWROILPANXX</t>
+          <t>PWROTHBTNXX</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>CO2PAN</t>
+          <t>CO2BTN</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.2077</v>
+        <v>0.0503</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2142,16 +2142,16 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PWROILPERXX</t>
+          <t>PWROTHINDEA</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>CO2PER</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.2177</v>
+        <v>0.0503</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2165,16 +2165,16 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PWROILPERXX</t>
+          <t>PWROTHINDEA</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>CO2PER</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0.2177</v>
+        <v>0.0503</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2188,16 +2188,16 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PWROILPRYXX</t>
+          <t>PWROTHINDNE</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>CO2PRY</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>0.2177</v>
+        <v>0.0503</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2211,16 +2211,16 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PWROILPRYXX</t>
+          <t>PWROTHINDNE</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>CO2PRY</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.2177</v>
+        <v>0.0503</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2234,16 +2234,16 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PWROILSLVXX</t>
+          <t>PWROTHINDNO</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>CO2SLV</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>0.1971</v>
+        <v>0.0503</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2257,16 +2257,16 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PWROILSLVXX</t>
+          <t>PWROTHINDNO</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>CO2SLV</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>0.1971</v>
+        <v>0.0503</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2280,16 +2280,16 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PWROILURYXX</t>
+          <t>PWROTHINDSO</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>CO2URY</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>0.2184</v>
+        <v>0.0503</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2303,16 +2303,16 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PWROILURYXX</t>
+          <t>PWROTHINDSO</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>CO2URY</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.2184</v>
+        <v>0.0503</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2326,16 +2326,16 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>PWRPETARGXX</t>
+          <t>PWROTHINDWE</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>CO2ARG</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.217</v>
+        <v>0.0503</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2349,16 +2349,16 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>PWRPETARGXX</t>
+          <t>PWROTHINDWE</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>CO2ARG</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>0.217</v>
+        <v>0.0503</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2372,16 +2372,16 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>PWRPETBOLXX</t>
+          <t>PWROTHLKAXX</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>CO2BOL</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>0.217</v>
+        <v>0.0503</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2395,16 +2395,16 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>PWRPETBOLXX</t>
+          <t>PWROTHLKAXX</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>CO2BOL</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>0.217</v>
+        <v>0.0503</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2418,16 +2418,16 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>PWRPETBRAXX</t>
+          <t>PWROTHNPLXX</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>CO2BRA</t>
+          <t>CO2NPL</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>0.217</v>
+        <v>0.0503</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2441,16 +2441,16 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>PWRPETBRAXX</t>
+          <t>PWROTHNPLXX</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>CO2BRA</t>
+          <t>CO2NPL</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0.217</v>
+        <v>0.0503</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2464,12 +2464,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>PWRPETBRBXX</t>
+          <t>PWRPETBGDXX</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>CO2BRB</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2487,12 +2487,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PWRPETBRBXX</t>
+          <t>PWRPETBGDXX</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>CO2BRB</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2510,12 +2510,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>PWRPETCHLXX</t>
+          <t>PWRPETBTNXX</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>CO2CHL</t>
+          <t>CO2BTN</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2533,12 +2533,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PWRPETCHLXX</t>
+          <t>PWRPETBTNXX</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>CO2CHL</t>
+          <t>CO2BTN</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2556,12 +2556,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>PWRPETCOLXX</t>
+          <t>PWRPETINDEA</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>CO2COL</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -2579,12 +2579,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>PWRPETCOLXX</t>
+          <t>PWRPETINDEA</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>CO2COL</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -2602,12 +2602,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>PWRPETCRIXX</t>
+          <t>PWRPETINDNE</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>CO2CRI</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -2625,12 +2625,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>PWRPETCRIXX</t>
+          <t>PWRPETINDNE</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>CO2CRI</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2648,12 +2648,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>PWRPETDOMXX</t>
+          <t>PWRPETINDNO</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>CO2DOM</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2671,12 +2671,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>PWRPETDOMXX</t>
+          <t>PWRPETINDNO</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>CO2DOM</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -2694,12 +2694,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PWRPETECUXX</t>
+          <t>PWRPETINDSO</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>CO2ECU</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2717,12 +2717,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>PWRPETECUXX</t>
+          <t>PWRPETINDSO</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>CO2ECU</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -2740,12 +2740,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>PWRPETGTMXX</t>
+          <t>PWRPETINDWE</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>CO2GTM</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -2763,12 +2763,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>PWRPETGTMXX</t>
+          <t>PWRPETINDWE</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>CO2GTM</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2786,12 +2786,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PWRPETHNDXX</t>
+          <t>PWRPETLKAXX</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>CO2HND</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2809,12 +2809,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>PWRPETHNDXX</t>
+          <t>PWRPETLKAXX</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>CO2HND</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2832,12 +2832,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>PWRPETHTIXX</t>
+          <t>PWRPETNPLXX</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>CO2HTI</t>
+          <t>CO2NPL</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -2855,12 +2855,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PWRPETHTIXX</t>
+          <t>PWRPETNPLXX</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>CO2HTI</t>
+          <t>CO2NPL</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -2878,16 +2878,16 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>PWRPETMEXXX</t>
+          <t>PWRWASBGDXX</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>CO2MEX</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>0.217</v>
+        <v>0.08790000000000001</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2897,20 +2897,20 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PWRPETMEXXX</t>
+          <t>PWRWASINDEA</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>CO2MEX</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.217</v>
+        <v>0.08790000000000001</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -2924,16 +2924,16 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>PWRPETNICXX</t>
+          <t>PWRWASINDNE</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>CO2NIC</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>0.217</v>
+        <v>0.08790000000000001</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -2943,20 +2943,20 @@
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>PWRPETNICXX</t>
+          <t>PWRWASINDNO</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>CO2NIC</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>0.217</v>
+        <v>0.08790000000000001</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -2970,16 +2970,16 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>PWRPETPANXX</t>
+          <t>PWRWASINDSO</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>CO2PAN</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>0.217</v>
+        <v>0.08790000000000001</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -2989,20 +2989,20 @@
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>PWRPETPANXX</t>
+          <t>PWRWASINDWE</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>CO2PAN</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0.217</v>
+        <v>0.08790000000000001</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3016,16 +3016,16 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>PWRPETPERXX</t>
+          <t>PWRWASLKAXX</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>CO2PER</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0.217</v>
+        <v>0.08790000000000001</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3035,597 +3035,22 @@
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>PWRPETPERXX</t>
+          <t>PWRWASNPLXX</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>CO2PER</t>
+          <t>CO2NPL</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>0.217</v>
+        <v>0.08790000000000001</v>
       </c>
       <c r="E113" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="n">
-        <v>1</v>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>PWRPETPRYXX</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>CO2PRY</t>
-        </is>
-      </c>
-      <c r="D114" t="n">
-        <v>0.217</v>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="n">
-        <v>2</v>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>PWRPETPRYXX</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>CO2PRY</t>
-        </is>
-      </c>
-      <c r="D115" t="n">
-        <v>0.217</v>
-      </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="n">
-        <v>1</v>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>PWRPETSLVXX</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>CO2SLV</t>
-        </is>
-      </c>
-      <c r="D116" t="n">
-        <v>0.217</v>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="n">
-        <v>2</v>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>PWRPETSLVXX</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>CO2SLV</t>
-        </is>
-      </c>
-      <c r="D117" t="n">
-        <v>0.217</v>
-      </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="n">
-        <v>1</v>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>PWRPETURYXX</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>CO2URY</t>
-        </is>
-      </c>
-      <c r="D118" t="n">
-        <v>0.217</v>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="n">
-        <v>2</v>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>PWRPETURYXX</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>CO2URY</t>
-        </is>
-      </c>
-      <c r="D119" t="n">
-        <v>0.217</v>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="n">
-        <v>1</v>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>PWRWASARGXX</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>CO2ARG</t>
-        </is>
-      </c>
-      <c r="D120" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="n">
-        <v>1</v>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>PWRWASBOLXX</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>CO2BOL</t>
-        </is>
-      </c>
-      <c r="D121" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="n">
-        <v>1</v>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>PWRWASBRAXX</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>CO2BRA</t>
-        </is>
-      </c>
-      <c r="D122" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="n">
-        <v>1</v>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>PWRWASBRBXX</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>CO2BRB</t>
-        </is>
-      </c>
-      <c r="D123" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="n">
-        <v>1</v>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>PWRWASCHLXX</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>CO2CHL</t>
-        </is>
-      </c>
-      <c r="D124" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="n">
-        <v>1</v>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>PWRWASCOLXX</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>CO2COL</t>
-        </is>
-      </c>
-      <c r="D125" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="n">
-        <v>1</v>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>PWRWASCRIXX</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>CO2CRI</t>
-        </is>
-      </c>
-      <c r="D126" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="n">
-        <v>1</v>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>PWRWASDOMXX</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>CO2DOM</t>
-        </is>
-      </c>
-      <c r="D127" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="n">
-        <v>1</v>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>PWRWASECUXX</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>CO2ECU</t>
-        </is>
-      </c>
-      <c r="D128" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="n">
-        <v>1</v>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>PWRWASGTMXX</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>CO2GTM</t>
-        </is>
-      </c>
-      <c r="D129" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="n">
-        <v>1</v>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>PWRWASHNDXX</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>CO2HND</t>
-        </is>
-      </c>
-      <c r="D130" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="n">
-        <v>1</v>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>PWRWASHTIXX</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>CO2HTI</t>
-        </is>
-      </c>
-      <c r="D131" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="n">
-        <v>1</v>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>PWRWASMEXXX</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>CO2MEX</t>
-        </is>
-      </c>
-      <c r="D132" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="n">
-        <v>1</v>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>PWRWASNICXX</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>CO2NIC</t>
-        </is>
-      </c>
-      <c r="D133" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="n">
-        <v>1</v>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>PWRWASPANXX</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>CO2PAN</t>
-        </is>
-      </c>
-      <c r="D134" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E134" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="n">
-        <v>1</v>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>PWRWASPERXX</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>CO2PER</t>
-        </is>
-      </c>
-      <c r="D135" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E135" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="n">
-        <v>1</v>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>PWRWASPRYXX</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>CO2PRY</t>
-        </is>
-      </c>
-      <c r="D136" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E136" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="n">
-        <v>1</v>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>PWRWASSLVXX</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>CO2SLV</t>
-        </is>
-      </c>
-      <c r="D137" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="n">
-        <v>1</v>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>PWRWASURYXX</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>CO2URY</t>
-        </is>
-      </c>
-      <c r="D138" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E138" t="inlineStr">
         <is>
           <t>MT</t>
         </is>

</xml_diff>

<commit_message>
Update model data inputs and outputs for MDV integration
</commit_message>
<xml_diff>
--- a/t1_confection/A2_Extra_Inputs/A-Xtra_Emissions.xlsx
+++ b/t1_confection/A2_Extra_Inputs/A-Xtra_Emissions.xlsx
@@ -1507,7 +1507,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.1292499999999999</v>
+        <v>0.12925</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1530,7 +1530,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.1292499999999999</v>
+        <v>0.12925</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update BAU model data for first Asia region
</commit_message>
<xml_diff>
--- a/t1_confection/A2_Extra_Inputs/A-Xtra_Emissions.xlsx
+++ b/t1_confection/A2_Extra_Inputs/A-Xtra_Emissions.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E115"/>
+  <dimension ref="A1:E111"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="19.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2372,12 +2372,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>PWROTHMDVXX</t>
+          <t>PWROTHNPLXX</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>CO2MDV</t>
+          <t>CO2NPL</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2395,12 +2395,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>PWROTHMDVXX</t>
+          <t>PWROTHNPLXX</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>CO2MDV</t>
+          <t>CO2NPL</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2418,16 +2418,16 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>PWROTHNPLXX</t>
+          <t>PWRPETBGDXX</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>CO2NPL</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>0.0503</v>
+        <v>0.217</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2441,16 +2441,16 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>PWROTHNPLXX</t>
+          <t>PWRPETBGDXX</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>CO2NPL</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0.0503</v>
+        <v>0.217</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2464,12 +2464,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>PWRPETBGDXX</t>
+          <t>PWRPETBTNXX</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>CO2BGD</t>
+          <t>CO2BTN</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2487,12 +2487,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PWRPETBGDXX</t>
+          <t>PWRPETBTNXX</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>CO2BGD</t>
+          <t>CO2BTN</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2510,12 +2510,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>PWRPETBTNXX</t>
+          <t>PWRPETINDEA</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>CO2BTN</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2533,12 +2533,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PWRPETBTNXX</t>
+          <t>PWRPETINDEA</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>CO2BTN</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>PWRPETINDEA</t>
+          <t>PWRPETINDNE</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>PWRPETINDEA</t>
+          <t>PWRPETINDNE</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>PWRPETINDNE</t>
+          <t>PWRPETINDNO</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>PWRPETINDNE</t>
+          <t>PWRPETINDNO</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2648,7 +2648,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>PWRPETINDNO</t>
+          <t>PWRPETINDSO</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2671,7 +2671,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>PWRPETINDNO</t>
+          <t>PWRPETINDSO</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PWRPETINDSO</t>
+          <t>PWRPETINDWE</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>PWRPETINDSO</t>
+          <t>PWRPETINDWE</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2740,12 +2740,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>PWRPETINDWE</t>
+          <t>PWRPETLKAXX</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>CO2IND</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -2763,12 +2763,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>PWRPETINDWE</t>
+          <t>PWRPETLKAXX</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>CO2IND</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2786,12 +2786,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PWRPETLKAXX</t>
+          <t>PWRPETNPLXX</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>CO2LKA</t>
+          <t>CO2NPL</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2809,12 +2809,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>PWRPETLKAXX</t>
+          <t>PWRPETNPLXX</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>CO2LKA</t>
+          <t>CO2NPL</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2832,16 +2832,16 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>PWRPETMDVXX</t>
+          <t>PWRWASBGDXX</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>CO2MDV</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0.217</v>
+        <v>0.08790000000000001</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2851,20 +2851,20 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PWRPETMDVXX</t>
+          <t>PWRWASINDEA</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>CO2MDV</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0.217</v>
+        <v>0.08790000000000001</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2878,16 +2878,16 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>PWRPETNPLXX</t>
+          <t>PWRWASINDNE</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>CO2NPL</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>0.217</v>
+        <v>0.08790000000000001</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2897,20 +2897,20 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PWRPETNPLXX</t>
+          <t>PWRWASINDNO</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>CO2NPL</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.217</v>
+        <v>0.08790000000000001</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -2924,12 +2924,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>PWRWASBGDXX</t>
+          <t>PWRWASINDSO</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>CO2BGD</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>PWRWASINDEA</t>
+          <t>PWRWASINDWE</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -2970,12 +2970,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>PWRWASINDNE</t>
+          <t>PWRWASLKAXX</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>CO2IND</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -2993,110 +2993,18 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>PWRWASINDNO</t>
+          <t>PWRWASNPLXX</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>CO2IND</t>
+          <t>CO2NPL</t>
         </is>
       </c>
       <c r="D111" t="n">
         <v>0.08790000000000001</v>
       </c>
       <c r="E111" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="n">
-        <v>1</v>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>PWRWASINDSO</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>CO2IND</t>
-        </is>
-      </c>
-      <c r="D112" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="n">
-        <v>1</v>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>PWRWASINDWE</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>CO2IND</t>
-        </is>
-      </c>
-      <c r="D113" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="n">
-        <v>1</v>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>PWRWASLKAXX</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>CO2LKA</t>
-        </is>
-      </c>
-      <c r="D114" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="n">
-        <v>1</v>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>PWRWASNPLXX</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>CO2NPL</t>
-        </is>
-      </c>
-      <c r="D115" t="n">
-        <v>0.08790000000000001</v>
-      </c>
-      <c r="E115" t="inlineStr">
         <is>
           <t>MT</t>
         </is>

</xml_diff>

<commit_message>
Update BAU model data: outputs, parameters, and input CSVs
</commit_message>
<xml_diff>
--- a/t1_confection/A2_Extra_Inputs/A-Xtra_Emissions.xlsx
+++ b/t1_confection/A2_Extra_Inputs/A-Xtra_Emissions.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E111"/>
+  <dimension ref="A1:E115"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="19.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2372,12 +2372,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>PWROTHNPLXX</t>
+          <t>PWROTHMDVXX</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>CO2NPL</t>
+          <t>CO2MDV</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2395,12 +2395,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>PWROTHNPLXX</t>
+          <t>PWROTHMDVXX</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>CO2NPL</t>
+          <t>CO2MDV</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2418,16 +2418,16 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>PWRPETBGDXX</t>
+          <t>PWROTHNPLXX</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>CO2BGD</t>
+          <t>CO2NPL</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>0.217</v>
+        <v>0.0503</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2441,16 +2441,16 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>PWRPETBGDXX</t>
+          <t>PWROTHNPLXX</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>CO2BGD</t>
+          <t>CO2NPL</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0.217</v>
+        <v>0.0503</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2464,12 +2464,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>PWRPETBTNXX</t>
+          <t>PWRPETBGDXX</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>CO2BTN</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2487,12 +2487,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PWRPETBTNXX</t>
+          <t>PWRPETBGDXX</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>CO2BTN</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2510,12 +2510,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>PWRPETINDEA</t>
+          <t>PWRPETBTNXX</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>CO2IND</t>
+          <t>CO2BTN</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2533,12 +2533,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PWRPETINDEA</t>
+          <t>PWRPETBTNXX</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>CO2IND</t>
+          <t>CO2BTN</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>PWRPETINDNE</t>
+          <t>PWRPETINDEA</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>PWRPETINDNE</t>
+          <t>PWRPETINDEA</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>PWRPETINDNO</t>
+          <t>PWRPETINDNE</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>PWRPETINDNO</t>
+          <t>PWRPETINDNE</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2648,7 +2648,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>PWRPETINDSO</t>
+          <t>PWRPETINDNO</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2671,7 +2671,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>PWRPETINDSO</t>
+          <t>PWRPETINDNO</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PWRPETINDWE</t>
+          <t>PWRPETINDSO</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>PWRPETINDWE</t>
+          <t>PWRPETINDSO</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2740,12 +2740,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>PWRPETLKAXX</t>
+          <t>PWRPETINDWE</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>CO2LKA</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -2763,12 +2763,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>PWRPETLKAXX</t>
+          <t>PWRPETINDWE</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>CO2LKA</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2786,12 +2786,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PWRPETNPLXX</t>
+          <t>PWRPETLKAXX</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>CO2NPL</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2809,12 +2809,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>PWRPETNPLXX</t>
+          <t>PWRPETLKAXX</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>CO2NPL</t>
+          <t>CO2LKA</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2832,16 +2832,16 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>PWRWASBGDXX</t>
+          <t>PWRPETMDVXX</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>CO2BGD</t>
+          <t>CO2MDV</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0.08790000000000001</v>
+        <v>0.217</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2851,20 +2851,20 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PWRWASINDEA</t>
+          <t>PWRPETMDVXX</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>CO2IND</t>
+          <t>CO2MDV</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0.08790000000000001</v>
+        <v>0.217</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2878,16 +2878,16 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>PWRWASINDNE</t>
+          <t>PWRPETNPLXX</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>CO2IND</t>
+          <t>CO2NPL</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>0.08790000000000001</v>
+        <v>0.217</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2897,20 +2897,20 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PWRWASINDNO</t>
+          <t>PWRPETNPLXX</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>CO2IND</t>
+          <t>CO2NPL</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.08790000000000001</v>
+        <v>0.217</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -2924,12 +2924,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>PWRWASINDSO</t>
+          <t>PWRWASBGDXX</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>CO2IND</t>
+          <t>CO2BGD</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>PWRWASINDWE</t>
+          <t>PWRWASINDEA</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -2970,12 +2970,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>PWRWASLKAXX</t>
+          <t>PWRWASINDNE</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>CO2LKA</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -2993,18 +2993,110 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>PWRWASNPLXX</t>
+          <t>PWRWASINDNO</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>CO2NPL</t>
+          <t>CO2IND</t>
         </is>
       </c>
       <c r="D111" t="n">
         <v>0.08790000000000001</v>
       </c>
       <c r="E111" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>1</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>PWRWASINDSO</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>CO2IND</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>0.08790000000000001</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>1</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>PWRWASINDWE</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>CO2IND</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>0.08790000000000001</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>1</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>PWRWASLKAXX</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>CO2LKA</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>0.08790000000000001</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>1</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>PWRWASNPLXX</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>CO2NPL</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>0.08790000000000001</v>
+      </c>
+      <c r="E115" t="inlineStr">
         <is>
           <t>MT</t>
         </is>

</xml_diff>